<commit_message>
feature: oops forgot to add mock data
</commit_message>
<xml_diff>
--- a/mockdata/AMRFinderPlus_Results.xlsx
+++ b/mockdata/AMRFinderPlus_Results.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="43">
   <si>
     <t>Isolate ID</t>
   </si>
@@ -19,13 +19,22 @@
     <t>Gene Symbol</t>
   </si>
   <si>
+    <t>Sequence Name</t>
+  </si>
+  <si>
     <t>Element Type</t>
   </si>
   <si>
-    <t>Resistance Class</t>
-  </si>
-  <si>
-    <t>Resistance Subclass</t>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Subclass</t>
+  </si>
+  <si>
+    <t>Target Length</t>
+  </si>
+  <si>
+    <t>Reference Length</t>
   </si>
   <si>
     <t>Identity %</t>
@@ -34,12 +43,21 @@
     <t>Coverage %</t>
   </si>
   <si>
+    <t>Alignment Length</t>
+  </si>
+  <si>
+    <t>Accession</t>
+  </si>
+  <si>
     <t>ISO-101</t>
   </si>
   <si>
     <t>bla</t>
   </si>
   <si>
+    <t>subclass B3 metallo-beta-lactamase</t>
+  </si>
+  <si>
     <t>AMR</t>
   </si>
   <si>
@@ -52,9 +70,15 @@
     <t>58.33</t>
   </si>
   <si>
+    <t>WP_122630833.1</t>
+  </si>
+  <si>
     <t>erm</t>
   </si>
   <si>
+    <t>23S rRNA methyltransferase Erm</t>
+  </si>
+  <si>
     <t>MACROLIDE</t>
   </si>
   <si>
@@ -64,12 +88,18 @@
     <t>39.76</t>
   </si>
   <si>
+    <t>WP_015345217.1</t>
+  </si>
+  <si>
     <t>ISO-102</t>
   </si>
   <si>
     <t>aac(3)-I</t>
   </si>
   <si>
+    <t>AAC(3)-I aminoglycoside</t>
+  </si>
+  <si>
     <t>AMINOGLYCOSIDE</t>
   </si>
   <si>
@@ -82,12 +112,18 @@
     <t>62.00</t>
   </si>
   <si>
+    <t>ABL71428.1</t>
+  </si>
+  <si>
     <t>ISO-103</t>
   </si>
   <si>
     <t>arsN1</t>
   </si>
   <si>
+    <t>arsinothricin N-acetyltransferase</t>
+  </si>
+  <si>
     <t>STRESS</t>
   </si>
   <si>
@@ -101,6 +137,9 @@
   </si>
   <si>
     <t>51.48</t>
+  </si>
+  <si>
+    <t>AAN67541.1</t>
   </si>
 </sst>
 </file>
@@ -122,6 +161,11 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
+      <sz val="15"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="12"/>
       <color indexed="9"/>
@@ -132,14 +176,8 @@
       <color indexed="9"/>
       <name val="Helvetica"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -152,109 +190,13 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="13"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="12"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="12"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="12"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="12"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="12"/>
-      </left>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -278,50 +220,29 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -344,8 +265,6 @@
       <rgbColor rgb="ff1f1f1f"/>
       <rgbColor rgb="ffefefef"/>
       <rgbColor rgb="ffa5a5a5"/>
-      <rgbColor rgb="ff3f3f3f"/>
-      <rgbColor rgb="ffdbdbdb"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -362,10 +281,10 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="5E5E5E"/>
+        <a:srgbClr val="A7A7A7"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="D5D5D5"/>
+        <a:srgbClr val="535353"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="00A2FF"/>
@@ -542,11 +461,14 @@
     <a:spDef>
       <a:spPr>
         <a:solidFill>
-          <a:srgbClr val="000000"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -555,33 +477,33 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="ctr" defTabSz="584200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
-          <a:lnSpc>
-            <a:spcPct val="100000"/>
-          </a:lnSpc>
-          <a:spcBef>
-            <a:spcPts val="0"/>
-          </a:spcBef>
-          <a:spcAft>
-            <a:spcPts val="0"/>
-          </a:spcAft>
-          <a:buClrTx/>
-          <a:buSzTx/>
-          <a:buFontTx/>
-          <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1200" u="none" kumimoji="0" normalizeH="0">
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:uFillTx/>
-            <a:latin typeface="Helvetica Neue Medium"/>
-            <a:ea typeface="Helvetica Neue Medium"/>
-            <a:cs typeface="Helvetica Neue Medium"/>
-            <a:sym typeface="Helvetica Neue Medium"/>
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -820,12 +742,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
-            <a:srgbClr val="000000"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="400000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1106,7 +1028,7 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="457200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
           <a:lnSpc>
             <a:spcPct val="100000"/>
           </a:lnSpc>
@@ -1374,11 +1296,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M22"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:O22"/>
+  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="13" width="16.3516" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col min="1" max="15" width="16.3516" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="16.3516" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="60.55" customHeight="1">
@@ -1403,383 +1325,477 @@
       <c r="G1" t="s" s="2">
         <v>6</v>
       </c>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
+      <c r="H1" t="s" s="2">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s" s="2">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s" s="2">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s" s="2">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s" s="2">
+        <v>11</v>
+      </c>
       <c r="M1" s="3"/>
-    </row>
-    <row r="2" ht="46.55" customHeight="1">
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+    </row>
+    <row r="2" ht="74.55" customHeight="1">
       <c r="A2" t="s" s="4">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s" s="5">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s" s="6">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s" s="6">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s" s="6">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s" s="6">
-        <v>11</v>
-      </c>
-      <c r="G2" t="s" s="6">
         <v>12</v>
       </c>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
+      <c r="B2" t="s" s="4">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s" s="4">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s" s="4">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s" s="4">
+        <v>16</v>
+      </c>
+      <c r="G2" s="5">
+        <v>278</v>
+      </c>
+      <c r="H2" s="5">
+        <v>295</v>
+      </c>
+      <c r="I2" t="s" s="4">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s" s="4">
+        <v>18</v>
+      </c>
+      <c r="K2" s="5">
+        <v>240</v>
+      </c>
+      <c r="L2" t="s" s="4">
+        <v>19</v>
+      </c>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
     </row>
     <row r="3" ht="46.35" customHeight="1">
-      <c r="A3" t="s" s="8">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s" s="9">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s" s="10">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s" s="10">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s" s="10">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s" s="10">
+      <c r="A3" t="s" s="4">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s" s="4">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s" s="4">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s" s="4">
         <v>15</v>
       </c>
-      <c r="G3" t="s" s="10">
-        <v>16</v>
-      </c>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
+      <c r="E3" t="s" s="4">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s" s="4">
+        <v>22</v>
+      </c>
+      <c r="G3" s="5">
+        <v>271</v>
+      </c>
+      <c r="H3" s="5">
+        <v>281</v>
+      </c>
+      <c r="I3" t="s" s="4">
+        <v>23</v>
+      </c>
+      <c r="J3" t="s" s="4">
+        <v>24</v>
+      </c>
+      <c r="K3" s="5">
+        <v>249</v>
+      </c>
+      <c r="L3" t="s" s="4">
+        <v>25</v>
+      </c>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
     </row>
     <row r="4" ht="60.35" customHeight="1">
-      <c r="A4" t="s" s="8">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s" s="9">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s" s="10">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s" s="10">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s" s="10">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s" s="10">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s" s="10">
-        <v>22</v>
-      </c>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
+      <c r="A4" t="s" s="4">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s" s="4">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s" s="4">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s" s="4">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s" s="4">
+        <v>29</v>
+      </c>
+      <c r="F4" t="s" s="4">
+        <v>30</v>
+      </c>
+      <c r="G4" s="5">
+        <v>196</v>
+      </c>
+      <c r="H4" s="5">
+        <v>152</v>
+      </c>
+      <c r="I4" t="s" s="4">
+        <v>31</v>
+      </c>
+      <c r="J4" t="s" s="4">
+        <v>32</v>
+      </c>
+      <c r="K4" s="5">
+        <v>150</v>
+      </c>
+      <c r="L4" t="s" s="4">
+        <v>33</v>
+      </c>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
     </row>
     <row r="5" ht="46.35" customHeight="1">
-      <c r="A5" t="s" s="8">
-        <v>23</v>
-      </c>
-      <c r="B5" t="s" s="9">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s" s="10">
-        <v>25</v>
-      </c>
-      <c r="D5" t="s" s="10">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s" s="10">
-        <v>27</v>
-      </c>
-      <c r="F5" t="s" s="10">
-        <v>28</v>
-      </c>
-      <c r="G5" t="s" s="10">
-        <v>29</v>
-      </c>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
+      <c r="A5" t="s" s="4">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s" s="4">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s" s="4">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s" s="4">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s" s="4">
+        <v>38</v>
+      </c>
+      <c r="F5" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="G5" s="5">
+        <v>202</v>
+      </c>
+      <c r="H5" s="5">
+        <v>186</v>
+      </c>
+      <c r="I5" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s" s="4">
+        <v>41</v>
+      </c>
+      <c r="K5" s="5">
+        <v>155</v>
+      </c>
+      <c r="L5" t="s" s="4">
+        <v>42</v>
+      </c>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
     </row>
     <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" s="13"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
     </row>
     <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
     </row>
     <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
     </row>
     <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
     </row>
     <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
     </row>
     <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
     </row>
     <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
     </row>
     <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
     </row>
     <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
     </row>
     <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="12"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
     </row>
     <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12"/>
-      <c r="M16" s="12"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
     </row>
     <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="12"/>
-      <c r="M17" s="12"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
     </row>
     <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
     </row>
     <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
-      <c r="M19" s="12"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="7"/>
     </row>
     <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
-      <c r="M20" s="12"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="7"/>
+      <c r="O20" s="7"/>
     </row>
     <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="12"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="7"/>
     </row>
     <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
-      <c r="M22" s="12"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>

</xml_diff>